<commit_message>
Unify comparison-table naming: YOLO11 → v11
Keep table version labels consistent with v1–v14 short form;
note Ultralytics product spelling separately in Excel cover sheet.

Co-authored-by: qidingdig <qidingdig@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/yolo-survey/tables/YOLO对比表.xlsx
+++ b/docs/yolo-survey/tables/YOLO对比表.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -524,31 +524,38 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>命名约定：表内统一 v1…v14 / v11；Ultralytics 产品原文常写作 YOLO11（无字母 v）。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>推荐用法</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>对内 Git 协作：CSV + Markdown；对外汇报/跨团队：本 xlsx；贴 PPT 前先复制数值区并注明来源。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>边界：表1不是精度排名；表2不是 COCO 官方总榜，且不含 v12+/YOLO26。</t>
+          <t>对内 Git 协作：CSV + Markdown；对外汇报/跨团队：本 xlsx；贴 PPT 前先复制数值区并注明来源。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>边界：表1不是精度排名；表2不是 COCO 官方总榜，且不含 v12+/YOLO26。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>生成日期：2026-07-28</t>
         </is>
@@ -831,7 +838,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>训练期存在辅助分支，训练计算更重；多任务一体化程度不及 v8/YOLO11</t>
+          <t>训练期存在辅助分支，训练计算更重；多任务一体化程度不及 v8/v11</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -875,7 +882,7 @@
     <row r="12" ht="55" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>YOLO11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1021,37 +1028,37 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv5</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv6</t>
+          <t>v6</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv7</t>
+          <t>v7</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv8</t>
+          <t>v8</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv9</t>
+          <t>v9</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv10</t>
+          <t>v10</t>
         </is>
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="J1" s="4" t="inlineStr">
@@ -1113,7 +1120,7 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -1170,7 +1177,7 @@
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr"/>
@@ -1223,7 +1230,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>YOLOv9</t>
+          <t>v9</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1280,7 +1287,7 @@
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr"/>
@@ -1333,7 +1340,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr"/>
@@ -1379,37 +1386,37 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv5</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv6</t>
+          <t>v6</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv7</t>
+          <t>v7</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv8</t>
+          <t>v8</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv9</t>
+          <t>v9</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv10</t>
+          <t>v10</t>
         </is>
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="J1" s="4" t="inlineStr">
@@ -1471,7 +1478,7 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr"/>
@@ -1524,7 +1531,7 @@
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr"/>
@@ -1577,7 +1584,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr"/>
@@ -1630,7 +1637,7 @@
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr"/>
@@ -1683,7 +1690,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>YOLOv9</t>
+          <t>v9</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr"/>
@@ -1736,7 +1743,7 @@
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>YOLOv9</t>
+          <t>v9</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr"/>
@@ -1789,7 +1796,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr"/>
@@ -1842,7 +1849,7 @@
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>YOLOv8</t>
+          <t>v8</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr"/>
@@ -1895,7 +1902,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>YOLOv8</t>
+          <t>v8</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr"/>
@@ -1948,7 +1955,7 @@
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>YOLOv5</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr"/>
@@ -2001,7 +2008,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr"/>
@@ -2047,37 +2054,37 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv5</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv6</t>
+          <t>v6</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv7</t>
+          <t>v7</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv8</t>
+          <t>v8</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv9</t>
+          <t>v9</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv10</t>
+          <t>v10</t>
         </is>
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="J1" s="4" t="inlineStr">
@@ -2139,7 +2146,7 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>YOLOv5</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -2196,7 +2203,7 @@
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>YOLOv5</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr"/>
@@ -2249,7 +2256,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>YOLOv9</t>
+          <t>v9</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr"/>
@@ -2302,7 +2309,7 @@
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>YOLOv8</t>
+          <t>v8</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr"/>
@@ -2355,7 +2362,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr"/>
@@ -2408,7 +2415,7 @@
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>YOLOv9</t>
+          <t>v9</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr"/>
@@ -2461,7 +2468,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr"/>
@@ -2514,7 +2521,7 @@
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>YOLOv8</t>
+          <t>v8</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr"/>
@@ -2567,7 +2574,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>YOLOv9</t>
+          <t>v9</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr"/>
@@ -2620,7 +2627,7 @@
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>YOLOv11</t>
+          <t>v11</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr"/>
@@ -2673,7 +2680,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>YOLOv9</t>
+          <t>v9</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Add v12/v13 paper COCO self-report comparison tables
Extract author-reported COCO tables from YOLOv12 and YOLOv13 papers
into CSV/Excel/Markdown, plus a cross-paper caution sheet so v12
numbers are not mixed across different source tables.

Co-authored-by: qidingdig <qidingdig@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/yolo-survey/tables/YOLO对比表.xlsx
+++ b/docs/yolo-survey/tables/YOLO对比表.xlsx
@@ -12,12 +12,18 @@
     <sheet name="表2a-ODverse33总体" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="表2b-分域mAP50" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="表2c-分域mAP50-95" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="表3-v12论文自报" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="表4-v13论文自报" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="表3-4速览" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'表1-机制演进对比'!$A$1:$E$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'表2a-ODverse33总体'!$A$1:$K$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'表2b-分域mAP50'!$A$1:$K$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'表2c-分域mAP50-95'!$A$1:$K$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'表3-v12论文自报'!$A$1:$J$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'表4-v13论文自报'!$A$1:$J$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'表3-4速览'!$A$1:$H$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,11 +45,6 @@
       <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -113,15 +114,15 @@
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -489,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -505,57 +506,61 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>表1：机制演进对比（v1–v14）——定性；来自 YOLO系列总表</t>
+          <t>表1：机制演进对比（v1–v14）——定性</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>表2a：ODverse33 总体指标（v5–v11）——定量；arXiv:2502.14314</t>
+          <t>表2：ODverse33 多域横比（v5–v11）——第三方统一协议</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>表2b：ODverse33 分域指标——定量；与表2a 同协议，勿与厂商 COCO 表混排</t>
+          <t>表3：v12 论文 COCO 自报（arXiv:2502.12524）</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>命名约定：表内统一 v1…v14 / v11；Ultralytics 产品原文常写作 YOLO11（无字母 v）。</t>
+          <t>表4：v13 论文 COCO 自报（arXiv:2506.17733）</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>表3-4速览：v11/v12/v13 同档对照 + 跨文数字差异提示</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>推荐用法</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>对内 Git 协作：CSV + Markdown；对外汇报/跨团队：本 xlsx；贴 PPT 前先复制数值区并注明来源。</t>
+          <t>命名：表内统一 v1…v14；厂商原文 YOLO11 无字母 v。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>边界：表1不是精度排名；表2不是 COCO 官方总榜，且不含 v12+/YOLO26。</t>
+          <t>规范：不同来源分 Sheet；勿把表3的v12与表4的v13直接拼绝对排名。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>v14：尚无完整公开 COCO 横表，未收录数值 Sheet。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>生成日期：2026-07-28</t>
         </is>
@@ -582,7 +587,7 @@
     <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>版本</t>
@@ -2689,4 +2694,2909 @@
   <autoFilter ref="A1:K12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>来源论文</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>档位</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>模型</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>FLOPs(G)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>参数(M)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>AP50-95</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>AP50</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>AP75</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Latency_T4_TRT_FP16(ms)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>v8</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>8.7</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>37.4</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>52.6</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>40.5</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>1.77</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>论文自报；640输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>v10</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>38.5</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>53.8</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>41.7</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>1.84</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>v11</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>55.3</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>42.8</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>v12</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>40.6</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>56.7</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>43.8</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>1.64</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>本文模型</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>v8</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>28.6</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>61.8</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>48.7</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>2.33</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>RT-DETR-R18</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>46.5</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>63.8</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>4.58</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>端到端对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>RT-DETRv2-R18</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>47.9</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>64.9</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>4.58</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>v9</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>26.4</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>46.8</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>63.4</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>50.7</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>v10</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>21.6</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>46.3</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>50.4</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>2.49</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>v11</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>21.5</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>46.9</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>63.9</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>50.6</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>v12</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>21.4</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>65.0</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>51.8</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>2.61</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>本文模型</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>v8</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>78.9</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>25.9</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>50.3</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>67.2</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>54.7</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>5.09</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>v9</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>76.3</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>51.4</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>68.1</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>56.1</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>v10</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>59.1</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>15.4</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>51.1</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>68.1</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>55.8</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>4.74</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>v11</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>20.1</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>51.5</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>68.5</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>55.7</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>v12</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>67.5</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>20.2</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>52.5</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>69.6</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>57.1</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>4.86</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>本文模型</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>v8</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>165.2</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>43.7</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>69.8</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>57.7</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>8.06</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>v9-c</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>102.1</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>25.3</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>70.2</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>57.8</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>v9 大档常用 c</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>v10</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>120.3</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>24.4</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>53.2</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>70.1</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>58.1</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>7.28</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>v11</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>86.9</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>25.3</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>53.3</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>70.1</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>58.2</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>v12</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>88.9</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>26.4</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>53.7</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>70.7</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>58.5</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>6.77</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>本文模型</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>v8</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>257.8</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>68.2</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>71.0</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>58.8</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>12.83</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>v10</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>160.4</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>29.5</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>71.3</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>59.3</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>10.70</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>v11</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>194.9</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>56.9</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>54.6</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>71.6</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>59.5</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2502.12524 Table1</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>v12</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>199.0</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>59.1</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>55.2</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>60.2</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>11.79</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>本文模型</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J26"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>来源论文</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>档位</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>模型</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>FLOPs(G)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>参数(M)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>AP50-95</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>AP50</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>AP75</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Latency_T4_TRT_FP16(ms)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>v8</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>8.7</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>37.4</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>52.6</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>40.5</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>1.77</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>论文自报；640；600 epoch 设定对齐叙述</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>v10</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>38.5</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>53.8</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>41.7</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>1.84</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>v11</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>38.6</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>54.2</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>41.6</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>与 v12 论文中的 v11-N(39.4) 不同源表，勿混排</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>v12</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>40.1</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>43.4</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>1.83</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>v13 文内复测/引用；低于 v12 原文 40.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>v13</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>6.4</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>41.6</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>57.8</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>45.1</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>1.97</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>本文模型；相对同表 v12-N +1.5 AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>v8</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>28.6</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>61.8</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>48.7</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>2.33</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>RT-DETRv2-R18</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>47.9</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>64.9</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>4.58</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>端到端对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>v9</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>26.4</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>46.8</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>63.4</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>50.7</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>3.44</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>v10</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>21.6</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>46.3</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>50.4</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>2.53</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>v11</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>21.5</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>45.8</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>62.6</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>49.8</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>2.56</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>v12</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>21.4</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>47.1</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>64.2</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>2.82</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>低于 v12 原文 48.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>v13</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>20.8</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>65.2</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>2.98</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>本文模型；相对同表 v12-S +0.9 AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>v8</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>165.2</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>43.7</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>69.8</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>57.7</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>8.13</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>v9-c</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>102.1</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>25.3</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>70.2</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>57.8</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>6.64</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>v10</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>120.3</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>24.4</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>53.2</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>70.1</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>57.2</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>7.31</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>v11</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>86.9</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>25.3</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>52.3</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>69.2</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>55.7</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>6.23</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>v12</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>88.9</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>26.4</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>57.9</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>7.10</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>低于 v12 原文 53.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>v13</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>88.4</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>27.6</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>70.9</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>58.1</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>8.63</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>本文模型；相对同表 v12-L +0.4 AP；延迟高于 v11/v12</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>v8</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>257.8</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>68.2</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>71.0</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>58.8</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>12.83</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>v10</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>160.4</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>29.5</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>71.3</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>59.3</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>10.70</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>v11</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>194.9</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>56.9</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>54.2</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>71.0</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>59.1</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>11.35</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>v12</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>199.0</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>59.1</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>71.1</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>59.3</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>12.46</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>低于 v12 原文 55.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>arXiv:2506.17733 TableI</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>v13</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>199.2</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>64.0</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>54.8</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>59.8</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>14.67</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>本文模型；相对同表 v12-X +0.4 AP；最慢</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J24"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>档位</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>指标</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>v11_出自v12文</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>v12_出自v12文</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>v11_出自v13文</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>v12_出自v13文</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>v13_出自v13文</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>阅读注意</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>AP50-95</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>40.6</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>38.6</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>40.1</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>41.6</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>两篇论文对同一对照模型数字不完全一致；同表内比相对增益，勿跨表拼绝对排名</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Latency_ms</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>1.64</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>1.83</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>1.97</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>T4 TensorRT FP16（各文自报）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>AP50-95</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>46.9</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>45.8</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>47.1</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Latency_ms</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>2.61</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>2.56</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>2.82</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>2.98</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>AP50-95</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>53.3</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>53.7</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>52.3</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>v13 无独立 m 档主表；此处用 l</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Latency_ms</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>6.77</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>6.23</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>7.10</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>8.63</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>v13-L 延迟明显高于 v11-L</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>AP50-95</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>54.6</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>55.2</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>54.2</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>54.8</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Latency_ms</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>11.79</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>11.35</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>12.46</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>14.67</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>v13-X 延迟最高</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>